<commit_message>
Style xlsx bar chart to match Word doc
Single navy series with value labels above each bar instead of Excel's
default one-color-per-row rendering.

https://claude.ai/code/session_01PM89wz7vnfvW2NRaFUoooy
</commit_message>
<xml_diff>
--- a/qr_weekly.xlsx
+++ b/qr_weekly.xlsx
@@ -168,10 +168,22 @@
             </strRef>
           </tx>
           <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="1F4E79"/>
+            </a:solidFill>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
+                <a:srgbClr val="1F4E79"/>
+              </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
+          <dLbls>
+            <showLegendKey val="0"/>
+            <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+          </dLbls>
           <cat>
             <numRef>
               <f>'Weekly QR Scans'!$A$2:$A$20</f>
@@ -183,10 +195,7 @@
             </numRef>
           </val>
         </ser>
-        <dLbls>
-          <showVal val="1"/>
-        </dLbls>
-        <gapWidth val="150"/>
+        <gapWidth val="60"/>
         <axId val="10"/>
         <axId val="100"/>
       </barChart>

</xml_diff>

<commit_message>
Render xlsx chart with wide bars and clean axes
Use text week labels so Excel picks the category axis (wide bars
instead of date-axis sticks), set major-unit ticks at 5, drop the
horizontal gridlines to match the doc's chart.

https://claude.ai/code/session_01PM89wz7vnfvW2NRaFUoooy
</commit_message>
<xml_diff>
--- a/qr_weekly.xlsx
+++ b/qr_weekly.xlsx
@@ -16,9 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -56,10 +54,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -195,7 +192,7 @@
             </numRef>
           </val>
         </ser>
-        <gapWidth val="60"/>
+        <gapWidth val="40"/>
         <axId val="10"/>
         <axId val="100"/>
       </barChart>
@@ -231,7 +228,6 @@
           <orientation val="minMax"/>
         </scaling>
         <axPos val="l"/>
-        <majorGridlines/>
         <title>
           <tx>
             <rich>
@@ -250,6 +246,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+        <majorUnit val="5"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
@@ -267,7 +264,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7920000" cy="3600000"/>
+    <ext cx="7920000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -577,7 +574,7 @@
   <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -594,152 +591,190 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>46041</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Jan 19</t>
+        </is>
       </c>
       <c r="B2" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>46048</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Jan 26</t>
+        </is>
       </c>
       <c r="B3" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>46055</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Feb 02</t>
+        </is>
       </c>
       <c r="B4" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>46062</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Feb 09</t>
+        </is>
       </c>
       <c r="B5" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>46069</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Feb 16</t>
+        </is>
       </c>
       <c r="B6" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>46076</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Feb 23</t>
+        </is>
       </c>
       <c r="B7" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>46083</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Mar 02</t>
+        </is>
       </c>
       <c r="B8" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>46090</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Mar 09</t>
+        </is>
       </c>
       <c r="B9" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
-        <v>46097</v>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Mar 16</t>
+        </is>
       </c>
       <c r="B10" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
-        <v>46104</v>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Mar 23</t>
+        </is>
       </c>
       <c r="B11" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>46111</v>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Mar 30</t>
+        </is>
       </c>
       <c r="B12" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>46118</v>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Apr 06</t>
+        </is>
       </c>
       <c r="B13" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>46125</v>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Apr 13</t>
+        </is>
       </c>
       <c r="B14" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>46132</v>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Apr 20</t>
+        </is>
       </c>
       <c r="B15" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n">
-        <v>46139</v>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Apr 27</t>
+        </is>
       </c>
       <c r="B16" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n">
-        <v>46146</v>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>May 04</t>
+        </is>
       </c>
       <c r="B17" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>46153</v>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>May 11</t>
+        </is>
       </c>
       <c r="B18" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n">
-        <v>46160</v>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>May 18</t>
+        </is>
       </c>
       <c r="B19" t="n">
         <v>27</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
-        <v>46167</v>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>May 25</t>
+        </is>
       </c>
       <c r="B20" t="n">
         <v>12</v>

</xml_diff>

<commit_message>
Show week-starting dates on xlsx chart x-axis
Drop the broken axis-title placeholders and force category labels to
render below the bars.

https://claude.ai/code/session_01PM89wz7vnfvW2NRaFUoooy
</commit_message>
<xml_diff>
--- a/qr_weekly.xlsx
+++ b/qr_weekly.xlsx
@@ -201,24 +201,11 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Week starting (Monday)</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="low"/>
         <crossAx val="100"/>
         <lblOffset val="100"/>
       </catAx>
@@ -227,22 +214,8 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>QR scans</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>

</xml_diff>

<commit_message>
Rotate xlsx x-axis labels and skip every other one
Match the SVG/Word doc look: dates angled ~30 degrees and only every
other week labelled to avoid crowding.

https://claude.ai/code/session_01PM89wz7vnfvW2NRaFUoooy
</commit_message>
<xml_diff>
--- a/qr_weekly.xlsx
+++ b/qr_weekly.xlsx
@@ -206,8 +206,20 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <tickLblPos val="low"/>
+        <txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-1800000" vert="horz"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="900"/>
+            </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
+          </a:p>
+        </txPr>
         <crossAx val="100"/>
         <lblOffset val="100"/>
+        <tickLblSkip val="2"/>
       </catAx>
       <valAx>
         <axId val="100"/>

</xml_diff>